<commit_message>
Initial commit: Inventory Management System with SQLite and Data Visualization
</commit_message>
<xml_diff>
--- a/inventory_report.xlsx
+++ b/inventory_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,16 @@
           <t>Minimum Stock</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total Stock Value (Cost)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Total Potential Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,12 +476,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>maize</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Grocery</t>
+          <t>grocery</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -490,6 +500,12 @@
       </c>
       <c r="H2" t="n">
         <v>20</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8100</v>
+      </c>
+      <c r="J2" t="n">
+        <v>9900</v>
       </c>
     </row>
     <row r="3">
@@ -520,10 +536,16 @@
         <v>380</v>
       </c>
       <c r="G3" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
       <c r="H3" t="n">
         <v>100</v>
+      </c>
+      <c r="I3" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>456000</v>
       </c>
     </row>
     <row r="4">
@@ -559,6 +581,12 @@
       <c r="H4" t="n">
         <v>50</v>
       </c>
+      <c r="I4" t="n">
+        <v>12500</v>
+      </c>
+      <c r="J4" t="n">
+        <v>17500</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -592,6 +620,52 @@
       </c>
       <c r="H5" t="n">
         <v>100</v>
+      </c>
+      <c r="I5" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>p005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>toothpaste</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>hygine</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F6" t="n">
+        <v>804</v>
+      </c>
+      <c r="G6" t="n">
+        <v>600</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>36000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>482400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>